<commit_message>
Updated POs till Feb
</commit_message>
<xml_diff>
--- a/FlightRisk/CustomerPrepayment.xlsx
+++ b/FlightRisk/CustomerPrepayment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leo/Github/XeroAPI/FlightRisk/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BED8E2-18B5-974C-B872-E8F78ABB6C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEA39AF-53AD-4247-B9F1-2A9F50A0DCF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9700" yWindow="-22820" windowWidth="27640" windowHeight="16520" xr2:uid="{38D5C541-7871-704C-ADD3-7E7071C154A8}"/>
+    <workbookView xWindow="6560" yWindow="-20980" windowWidth="27640" windowHeight="16520" xr2:uid="{38D5C541-7871-704C-ADD3-7E7071C154A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Sales Order Number</t>
   </si>
@@ -47,25 +47,136 @@
     <t>Prepayment $</t>
   </si>
   <si>
-    <t>FRC#2637</t>
-  </si>
-  <si>
-    <t>FRC#3130</t>
-  </si>
-  <si>
     <t>FRC#3194</t>
   </si>
   <si>
-    <t>FRC#3197</t>
-  </si>
-  <si>
-    <t>SI-00000547</t>
-  </si>
-  <si>
-    <t>SI-00000580</t>
-  </si>
-  <si>
-    <t>FRC#3917</t>
+    <t>FRC#3444</t>
+  </si>
+  <si>
+    <t>FRC#3499</t>
+  </si>
+  <si>
+    <t>FRC#3548</t>
+  </si>
+  <si>
+    <t>FRC#3549</t>
+  </si>
+  <si>
+    <t>FRC#3585</t>
+  </si>
+  <si>
+    <t>FRC#3615</t>
+  </si>
+  <si>
+    <t>FRC#3617</t>
+  </si>
+  <si>
+    <t>FRC#3626</t>
+  </si>
+  <si>
+    <t>FRC#3627</t>
+  </si>
+  <si>
+    <t>FRC#3636</t>
+  </si>
+  <si>
+    <t>FRC#3641</t>
+  </si>
+  <si>
+    <t>FRC#3649</t>
+  </si>
+  <si>
+    <t>FRC#3651</t>
+  </si>
+  <si>
+    <t>FRC#3657</t>
+  </si>
+  <si>
+    <t>FRC#3659</t>
+  </si>
+  <si>
+    <t>FRC#3661</t>
+  </si>
+  <si>
+    <t>FRC#3662</t>
+  </si>
+  <si>
+    <t>FRC#3663</t>
+  </si>
+  <si>
+    <t>FRC#3675</t>
+  </si>
+  <si>
+    <t>FRC#3676</t>
+  </si>
+  <si>
+    <t>FRC#3678</t>
+  </si>
+  <si>
+    <t>FRC#3680</t>
+  </si>
+  <si>
+    <t>FRC#3683</t>
+  </si>
+  <si>
+    <t>FRC#3684</t>
+  </si>
+  <si>
+    <t>FRC#3686</t>
+  </si>
+  <si>
+    <t>FRC#3688</t>
+  </si>
+  <si>
+    <t>FRC#3698</t>
+  </si>
+  <si>
+    <t>FRC#3702</t>
+  </si>
+  <si>
+    <t>FRC#3704</t>
+  </si>
+  <si>
+    <t>FRC#3716</t>
+  </si>
+  <si>
+    <t>FRC#3747</t>
+  </si>
+  <si>
+    <t>SI-00000694</t>
+  </si>
+  <si>
+    <t>SI-00000734</t>
+  </si>
+  <si>
+    <t>SI-00000738</t>
+  </si>
+  <si>
+    <t>SI-00000751</t>
+  </si>
+  <si>
+    <t>SI-00000752</t>
+  </si>
+  <si>
+    <t>SI-00000753</t>
+  </si>
+  <si>
+    <t>SI-00000754</t>
+  </si>
+  <si>
+    <t>SI-00000755</t>
+  </si>
+  <si>
+    <t>SI-00000771</t>
+  </si>
+  <si>
+    <t>SI-00000807</t>
+  </si>
+  <si>
+    <t>SI-00000808</t>
+  </si>
+  <si>
+    <t>SI-00000809</t>
   </si>
 </sst>
 </file>
@@ -454,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43792BBA-C766-5C40-9C57-A0361E6015E8}">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -473,10 +584,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>45990</v>
+        <v>46020</v>
       </c>
       <c r="C2" s="4">
-        <v>4508.99</v>
+        <v>11635.98</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -484,10 +595,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>46017</v>
+        <v>46037</v>
       </c>
       <c r="C3" s="4">
-        <v>4248.99</v>
+        <v>2958.98</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -495,10 +606,10 @@
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>46020</v>
+        <v>46042</v>
       </c>
       <c r="C4" s="4">
-        <v>11635.98</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -506,229 +617,451 @@
         <v>6</v>
       </c>
       <c r="B5" s="3">
-        <v>46022</v>
-      </c>
-      <c r="C5" s="2">
-        <v>799</v>
+        <v>46043</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3983.99</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3">
-        <v>46021</v>
-      </c>
-      <c r="C6" s="2">
-        <v>-799</v>
+        <v>46043</v>
+      </c>
+      <c r="C6" s="4">
+        <v>4399</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3">
-        <v>46013</v>
+        <v>46045</v>
       </c>
       <c r="C7" s="4">
-        <v>20242.47</v>
+        <v>2848.99</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3">
-        <v>46020</v>
-      </c>
-      <c r="C8" s="4">
-        <v>11021.99</v>
+        <v>46049</v>
+      </c>
+      <c r="C8" s="2">
+        <v>294.95999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="4"/>
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2799</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C10" s="2">
+        <v>259.98</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="4"/>
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C11" s="4">
+        <v>2579.09</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C12" s="4">
+        <v>3983.99</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="4"/>
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C13" s="4">
+        <v>3333.23</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
+      <c r="A14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C14" s="2">
+        <v>149.99</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
+      <c r="A15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C15" s="4">
+        <v>2783.99</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1999</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
+      <c r="A17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C17" s="4">
+        <v>2783.99</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
+      <c r="A18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C18" s="4">
+        <v>2916.99</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="4"/>
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C19" s="4">
+        <v>2399</v>
+      </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
+      <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C20" s="4">
+        <v>4048.99</v>
+      </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="4"/>
+      <c r="A21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C21" s="4">
+        <v>3999</v>
+      </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="2"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="4"/>
+      <c r="A22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C22" s="4">
+        <v>2798.99</v>
+      </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="2"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="4"/>
+      <c r="A23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C23" s="2">
+        <v>79.989999999999995</v>
+      </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="4"/>
+      <c r="A24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46053</v>
+      </c>
+      <c r="C24" s="4">
+        <v>1999</v>
+      </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="4"/>
+      <c r="A25" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C25" s="4">
+        <v>3999</v>
+      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="2"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="4"/>
+      <c r="A26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C26" s="4">
+        <v>3608.99</v>
+      </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="4"/>
+      <c r="A27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C27" s="4">
+        <v>3499</v>
+      </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="4"/>
+      <c r="A28" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C28" s="4">
+        <v>3999</v>
+      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="4"/>
+      <c r="A29" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C29" s="4">
+        <v>2699</v>
+      </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="2"/>
+      <c r="A30" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C30" s="4">
+        <v>4083.99</v>
+      </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="4"/>
+      <c r="A31" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46049</v>
+      </c>
+      <c r="C31" s="4">
+        <v>4373.96</v>
+      </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="2"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="4"/>
+      <c r="A32" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46052</v>
+      </c>
+      <c r="C32" s="4">
+        <v>4248.9799999999996</v>
+      </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="2"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="4"/>
+      <c r="A33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46053</v>
+      </c>
+      <c r="C33" s="4">
+        <v>2699</v>
+      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="2"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="4"/>
+      <c r="A34" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="3">
+        <v>46041</v>
+      </c>
+      <c r="C34" s="4">
+        <v>10722.76</v>
+      </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="2"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
+      <c r="A35" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46048</v>
+      </c>
+      <c r="C35" s="4">
+        <v>7047.75</v>
+      </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="2"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="4"/>
+      <c r="A36" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46048</v>
+      </c>
+      <c r="C36" s="4">
+        <v>9071.98</v>
+      </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="2"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="4"/>
+      <c r="A37" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C37" s="4">
+        <v>23390.22</v>
+      </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="2"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="4"/>
+      <c r="A38" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C38" s="4">
+        <v>2999.25</v>
+      </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="2"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="4"/>
+      <c r="A39" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C39" s="4">
+        <v>2999.25</v>
+      </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="2"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="4"/>
+      <c r="A40" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C40" s="4">
+        <v>2999.25</v>
+      </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="2"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="4"/>
+      <c r="A41" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="3">
+        <v>46050</v>
+      </c>
+      <c r="C41" s="4">
+        <v>7047.74</v>
+      </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="2"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="4"/>
+      <c r="A42" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="3">
+        <v>46052</v>
+      </c>
+      <c r="C42" s="4">
+        <v>8226</v>
+      </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="2"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="4"/>
+      <c r="A43" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" s="3">
+        <v>46053</v>
+      </c>
+      <c r="C43" s="4">
+        <v>1499.25</v>
+      </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="2"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="4"/>
+      <c r="A44" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44" s="3">
+        <v>46053</v>
+      </c>
+      <c r="C44" s="4">
+        <v>4497.75</v>
+      </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="2"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="4"/>
+      <c r="A45" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="3">
+        <v>46051</v>
+      </c>
+      <c r="C45" s="4">
+        <v>2999.25</v>
+      </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
@@ -743,12 +1076,12 @@
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="3"/>
-      <c r="C48" s="4"/>
+      <c r="C48" s="2"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="3"/>
-      <c r="C49" s="4"/>
+      <c r="C49" s="2"/>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
@@ -763,12 +1096,12 @@
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="3"/>
-      <c r="C52" s="2"/>
+      <c r="C52" s="4"/>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="3"/>
-      <c r="C53" s="2"/>
+      <c r="C53" s="4"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
@@ -828,7 +1161,7 @@
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="3"/>
-      <c r="C65" s="4"/>
+      <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
@@ -838,7 +1171,7 @@
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="3"/>
-      <c r="C67" s="2"/>
+      <c r="C67" s="4"/>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
@@ -898,7 +1231,7 @@
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="3"/>
-      <c r="C79" s="4"/>
+      <c r="C79" s="2"/>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
@@ -908,7 +1241,7 @@
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="3"/>
-      <c r="C81" s="2"/>
+      <c r="C81" s="4"/>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
@@ -943,7 +1276,7 @@
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="3"/>
-      <c r="C88" s="4"/>
+      <c r="C88" s="2"/>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
@@ -953,17 +1286,7 @@
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="3"/>
-      <c r="C90" s="2"/>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="2"/>
-      <c r="B91" s="3"/>
-      <c r="C91" s="4"/>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" s="2"/>
-      <c r="B92" s="3"/>
-      <c r="C92" s="4"/>
+      <c r="C90" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>